<commit_message>
Move Photos folder into Project
</commit_message>
<xml_diff>
--- a/Session 20/Ứng dụng Ecommerce.xlsx
+++ b/Session 20/Ứng dụng Ecommerce.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/fdfa2ef0cba258be/Desktop/Rikkei/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/FDFA2EF0CBA258BE/Desktop/Rikkei/Module 1/Session 20/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="11_50513C555653DBEF8F7D44ED0466E0F7582BC4AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5DC52310-86C5-46D2-A193-F438AC1F75AA}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="11_50513C555653DBEF8F7D44ED0466E0F7582BC4AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{45D6F713-A54A-4E69-A2DF-7870D6E40D6D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Danh sách task" sheetId="1" r:id="rId1"/>
@@ -819,45 +819,19 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -876,6 +850,8 @@
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -898,9 +874,33 @@
     <xf numFmtId="0" fontId="5" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
@@ -1025,10 +1025,6 @@
     <xdr:clientData fLocksWithSheet="0"/>
   </xdr:oneCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1251,50 +1247,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="80" t="s">
+      <c r="A1" s="82" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="80" t="s">
+      <c r="B1" s="82" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="80" t="s">
+      <c r="C1" s="82" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="92" t="s">
+      <c r="D1" s="112" t="s">
         <v>89</v>
       </c>
-      <c r="E1" s="80" t="s">
+      <c r="E1" s="82" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="80" t="s">
+      <c r="F1" s="82" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="94" t="s">
+      <c r="G1" s="114" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="95"/>
-      <c r="I1" s="95"/>
-      <c r="J1" s="95"/>
-      <c r="K1" s="95"/>
-      <c r="L1" s="95"/>
-      <c r="M1" s="95"/>
-      <c r="N1" s="96"/>
-      <c r="O1" s="80" t="s">
+      <c r="H1" s="81"/>
+      <c r="I1" s="81"/>
+      <c r="J1" s="81"/>
+      <c r="K1" s="81"/>
+      <c r="L1" s="81"/>
+      <c r="M1" s="81"/>
+      <c r="N1" s="115"/>
+      <c r="O1" s="82" t="s">
         <v>6</v>
       </c>
-      <c r="P1" s="80" t="s">
+      <c r="P1" s="82" t="s">
         <v>7</v>
       </c>
-      <c r="Q1" s="80" t="s">
+      <c r="Q1" s="82" t="s">
         <v>8</v>
       </c>
-      <c r="R1" s="80" t="s">
+      <c r="R1" s="82" t="s">
         <v>9</v>
       </c>
-      <c r="S1" s="80" t="s">
+      <c r="S1" s="82" t="s">
         <v>10</v>
       </c>
-      <c r="T1" s="80" t="s">
+      <c r="T1" s="82" t="s">
         <v>11</v>
       </c>
       <c r="U1" s="1"/>
@@ -1306,12 +1302,12 @@
       <c r="AA1" s="1"/>
     </row>
     <row r="2" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="81"/>
-      <c r="B2" s="81"/>
-      <c r="C2" s="81"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="81"/>
-      <c r="F2" s="81"/>
+      <c r="A2" s="83"/>
+      <c r="B2" s="83"/>
+      <c r="C2" s="83"/>
+      <c r="D2" s="113"/>
+      <c r="E2" s="83"/>
+      <c r="F2" s="83"/>
       <c r="G2" s="2" t="s">
         <v>12</v>
       </c>
@@ -1336,12 +1332,12 @@
       <c r="N2" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="O2" s="81"/>
-      <c r="P2" s="81"/>
-      <c r="Q2" s="81"/>
-      <c r="R2" s="81"/>
-      <c r="S2" s="81"/>
-      <c r="T2" s="81"/>
+      <c r="O2" s="83"/>
+      <c r="P2" s="83"/>
+      <c r="Q2" s="83"/>
+      <c r="R2" s="83"/>
+      <c r="S2" s="83"/>
+      <c r="T2" s="83"/>
       <c r="U2" s="1"/>
       <c r="V2" s="1"/>
       <c r="W2" s="1"/>
@@ -1351,7 +1347,7 @@
       <c r="AA2" s="1"/>
     </row>
     <row r="3" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="82" t="s">
+      <c r="A3" s="108" t="s">
         <v>20</v>
       </c>
       <c r="B3" s="18" t="s">
@@ -1392,8 +1388,8 @@
       <c r="AA3" s="27"/>
     </row>
     <row r="4" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="83"/>
-      <c r="B4" s="98" t="s">
+      <c r="A4" s="85"/>
+      <c r="B4" s="84" t="s">
         <v>25</v>
       </c>
       <c r="C4" s="79" t="s">
@@ -1431,8 +1427,8 @@
       <c r="AA4" s="27"/>
     </row>
     <row r="5" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="83"/>
-      <c r="B5" s="83"/>
+      <c r="A5" s="85"/>
+      <c r="B5" s="85"/>
       <c r="C5" s="79" t="s">
         <v>27</v>
       </c>
@@ -1468,8 +1464,8 @@
       <c r="AA5" s="27"/>
     </row>
     <row r="6" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="83"/>
-      <c r="B6" s="83"/>
+      <c r="A6" s="85"/>
+      <c r="B6" s="85"/>
       <c r="C6" s="79" t="s">
         <v>28</v>
       </c>
@@ -1505,8 +1501,8 @@
       <c r="AA6" s="27"/>
     </row>
     <row r="7" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="83"/>
-      <c r="B7" s="83"/>
+      <c r="A7" s="85"/>
+      <c r="B7" s="85"/>
       <c r="C7" s="79" t="s">
         <v>29</v>
       </c>
@@ -1542,8 +1538,8 @@
       <c r="AA7" s="27"/>
     </row>
     <row r="8" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="83"/>
-      <c r="B8" s="83"/>
+      <c r="A8" s="85"/>
+      <c r="B8" s="85"/>
       <c r="C8" s="79" t="s">
         <v>30</v>
       </c>
@@ -1579,8 +1575,8 @@
       <c r="AA8" s="27"/>
     </row>
     <row r="9" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="83"/>
-      <c r="B9" s="83"/>
+      <c r="A9" s="85"/>
+      <c r="B9" s="85"/>
       <c r="C9" s="79" t="s">
         <v>31</v>
       </c>
@@ -1616,8 +1612,8 @@
       <c r="AA9" s="27"/>
     </row>
     <row r="10" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="83"/>
-      <c r="B10" s="84"/>
+      <c r="A10" s="85"/>
+      <c r="B10" s="86"/>
       <c r="C10" s="79" t="s">
         <v>32</v>
       </c>
@@ -1653,8 +1649,8 @@
       <c r="AA10" s="27"/>
     </row>
     <row r="11" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="83"/>
-      <c r="B11" s="85" t="s">
+      <c r="A11" s="85"/>
+      <c r="B11" s="109" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="79" t="s">
@@ -1692,8 +1688,8 @@
       <c r="AA11" s="27"/>
     </row>
     <row r="12" spans="1:27" s="28" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="84"/>
-      <c r="B12" s="84"/>
+      <c r="A12" s="86"/>
+      <c r="B12" s="86"/>
       <c r="C12" s="79" t="s">
         <v>35</v>
       </c>
@@ -1729,7 +1725,7 @@
       <c r="AA12" s="27"/>
     </row>
     <row r="13" spans="1:27" s="43" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="99" t="s">
+      <c r="A13" s="87" t="s">
         <v>36</v>
       </c>
       <c r="B13" s="32" t="s">
@@ -1772,8 +1768,8 @@
       <c r="AA13" s="42"/>
     </row>
     <row r="14" spans="1:27" s="43" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="100"/>
-      <c r="B14" s="102" t="s">
+      <c r="A14" s="88"/>
+      <c r="B14" s="90" t="s">
         <v>25</v>
       </c>
       <c r="C14" s="79" t="s">
@@ -1811,8 +1807,8 @@
       <c r="AA14" s="42"/>
     </row>
     <row r="15" spans="1:27" s="43" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="100"/>
-      <c r="B15" s="100"/>
+      <c r="A15" s="88"/>
+      <c r="B15" s="88"/>
       <c r="C15" s="79" t="s">
         <v>29</v>
       </c>
@@ -1848,8 +1844,8 @@
       <c r="AA15" s="42"/>
     </row>
     <row r="16" spans="1:27" s="43" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="100"/>
-      <c r="B16" s="101"/>
+      <c r="A16" s="88"/>
+      <c r="B16" s="89"/>
       <c r="C16" s="79" t="s">
         <v>38</v>
       </c>
@@ -1885,7 +1881,7 @@
       <c r="AA16" s="42"/>
     </row>
     <row r="17" spans="1:27" s="43" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="101"/>
+      <c r="A17" s="89"/>
       <c r="B17" s="32" t="s">
         <v>39</v>
       </c>
@@ -1924,10 +1920,10 @@
       <c r="AA17" s="42"/>
     </row>
     <row r="18" spans="1:27" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="103" t="s">
+      <c r="A18" s="91" t="s">
         <v>41</v>
       </c>
-      <c r="B18" s="105" t="s">
+      <c r="B18" s="93" t="s">
         <v>33</v>
       </c>
       <c r="C18" s="79" t="s">
@@ -1965,8 +1961,8 @@
       <c r="AA18" s="55"/>
     </row>
     <row r="19" spans="1:27" s="56" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="104"/>
-      <c r="B19" s="104"/>
+      <c r="A19" s="92"/>
+      <c r="B19" s="92"/>
       <c r="C19" s="79" t="s">
         <v>43</v>
       </c>
@@ -2002,10 +1998,10 @@
       <c r="AA19" s="55"/>
     </row>
     <row r="20" spans="1:27" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="86" t="s">
+      <c r="A20" s="110" t="s">
         <v>44</v>
       </c>
-      <c r="B20" s="106" t="s">
+      <c r="B20" s="94" t="s">
         <v>45</v>
       </c>
       <c r="C20" s="17" t="s">
@@ -2043,8 +2039,8 @@
       <c r="AA20" s="64"/>
     </row>
     <row r="21" spans="1:27" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="87"/>
-      <c r="B21" s="87"/>
+      <c r="A21" s="95"/>
+      <c r="B21" s="95"/>
       <c r="C21" s="17" t="s">
         <v>47</v>
       </c>
@@ -2080,8 +2076,8 @@
       <c r="AA21" s="64"/>
     </row>
     <row r="22" spans="1:27" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="87"/>
-      <c r="B22" s="87"/>
+      <c r="A22" s="95"/>
+      <c r="B22" s="95"/>
       <c r="C22" s="17" t="s">
         <v>48</v>
       </c>
@@ -2117,8 +2113,8 @@
       <c r="AA22" s="64"/>
     </row>
     <row r="23" spans="1:27" s="65" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="88"/>
-      <c r="B23" s="88"/>
+      <c r="A23" s="96"/>
+      <c r="B23" s="96"/>
       <c r="C23" s="17" t="s">
         <v>49</v>
       </c>
@@ -2154,10 +2150,10 @@
       <c r="AA23" s="64"/>
     </row>
     <row r="24" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="89" t="s">
+      <c r="A24" s="111" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="109" t="s">
+      <c r="B24" s="99" t="s">
         <v>45</v>
       </c>
       <c r="C24" s="17" t="s">
@@ -2195,8 +2191,8 @@
       <c r="AA24" s="74"/>
     </row>
     <row r="25" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="90"/>
-      <c r="B25" s="110"/>
+      <c r="A25" s="105"/>
+      <c r="B25" s="100"/>
       <c r="C25" s="17" t="s">
         <v>52</v>
       </c>
@@ -2232,8 +2228,8 @@
       <c r="AA25" s="74"/>
     </row>
     <row r="26" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="90"/>
-      <c r="B26" s="110"/>
+      <c r="A26" s="105"/>
+      <c r="B26" s="100"/>
       <c r="C26" s="17" t="s">
         <v>53</v>
       </c>
@@ -2269,8 +2265,8 @@
       <c r="AA26" s="74"/>
     </row>
     <row r="27" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="90"/>
-      <c r="B27" s="110"/>
+      <c r="A27" s="105"/>
+      <c r="B27" s="100"/>
       <c r="C27" s="17" t="s">
         <v>54</v>
       </c>
@@ -2306,8 +2302,8 @@
       <c r="AA27" s="74"/>
     </row>
     <row r="28" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="90"/>
-      <c r="B28" s="111"/>
+      <c r="A28" s="105"/>
+      <c r="B28" s="101"/>
       <c r="C28" s="17" t="s">
         <v>55</v>
       </c>
@@ -2343,8 +2339,8 @@
       <c r="AA28" s="74"/>
     </row>
     <row r="29" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="90"/>
-      <c r="B29" s="109" t="s">
+      <c r="A29" s="105"/>
+      <c r="B29" s="99" t="s">
         <v>56</v>
       </c>
       <c r="C29" s="17" t="s">
@@ -2382,8 +2378,8 @@
       <c r="AA29" s="74"/>
     </row>
     <row r="30" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="90"/>
-      <c r="B30" s="110"/>
+      <c r="A30" s="105"/>
+      <c r="B30" s="100"/>
       <c r="C30" s="17" t="s">
         <v>58</v>
       </c>
@@ -2419,8 +2415,8 @@
       <c r="AA30" s="74"/>
     </row>
     <row r="31" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="90"/>
-      <c r="B31" s="110"/>
+      <c r="A31" s="105"/>
+      <c r="B31" s="100"/>
       <c r="C31" s="17" t="s">
         <v>59</v>
       </c>
@@ -2456,8 +2452,8 @@
       <c r="AA31" s="74"/>
     </row>
     <row r="32" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="90"/>
-      <c r="B32" s="110"/>
+      <c r="A32" s="105"/>
+      <c r="B32" s="100"/>
       <c r="C32" s="17" t="s">
         <v>60</v>
       </c>
@@ -2493,8 +2489,8 @@
       <c r="AA32" s="74"/>
     </row>
     <row r="33" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="90"/>
-      <c r="B33" s="111"/>
+      <c r="A33" s="105"/>
+      <c r="B33" s="101"/>
       <c r="C33" s="17" t="s">
         <v>61</v>
       </c>
@@ -2530,8 +2526,8 @@
       <c r="AA33" s="74"/>
     </row>
     <row r="34" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="90"/>
-      <c r="B34" s="112" t="s">
+      <c r="A34" s="105"/>
+      <c r="B34" s="102" t="s">
         <v>62</v>
       </c>
       <c r="C34" s="17" t="s">
@@ -2569,8 +2565,8 @@
       <c r="AA34" s="74"/>
     </row>
     <row r="35" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="90"/>
-      <c r="B35" s="113"/>
+      <c r="A35" s="105"/>
+      <c r="B35" s="103"/>
       <c r="C35" s="17" t="s">
         <v>64</v>
       </c>
@@ -2606,8 +2602,8 @@
       <c r="AA35" s="74"/>
     </row>
     <row r="36" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="90"/>
-      <c r="B36" s="114"/>
+      <c r="A36" s="105"/>
+      <c r="B36" s="104"/>
       <c r="C36" s="17" t="s">
         <v>65</v>
       </c>
@@ -2643,8 +2639,8 @@
       <c r="AA36" s="74"/>
     </row>
     <row r="37" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="90"/>
-      <c r="B37" s="112" t="s">
+      <c r="A37" s="105"/>
+      <c r="B37" s="102" t="s">
         <v>66</v>
       </c>
       <c r="C37" s="17" t="s">
@@ -2682,8 +2678,8 @@
       <c r="AA37" s="74"/>
     </row>
     <row r="38" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="90"/>
-      <c r="B38" s="90"/>
+      <c r="A38" s="105"/>
+      <c r="B38" s="105"/>
       <c r="C38" s="17" t="s">
         <v>68</v>
       </c>
@@ -2719,8 +2715,8 @@
       <c r="AA38" s="74"/>
     </row>
     <row r="39" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="90"/>
-      <c r="B39" s="91"/>
+      <c r="A39" s="105"/>
+      <c r="B39" s="106"/>
       <c r="C39" s="17" t="s">
         <v>69</v>
       </c>
@@ -2756,8 +2752,8 @@
       <c r="AA39" s="74"/>
     </row>
     <row r="40" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="90"/>
-      <c r="B40" s="112" t="s">
+      <c r="A40" s="105"/>
+      <c r="B40" s="102" t="s">
         <v>70</v>
       </c>
       <c r="C40" s="17" t="s">
@@ -2795,8 +2791,8 @@
       <c r="AA40" s="74"/>
     </row>
     <row r="41" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="90"/>
-      <c r="B41" s="90"/>
+      <c r="A41" s="105"/>
+      <c r="B41" s="105"/>
       <c r="C41" s="17" t="s">
         <v>72</v>
       </c>
@@ -2832,8 +2828,8 @@
       <c r="AA41" s="74"/>
     </row>
     <row r="42" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="90"/>
-      <c r="B42" s="90"/>
+      <c r="A42" s="105"/>
+      <c r="B42" s="105"/>
       <c r="C42" s="17" t="s">
         <v>73</v>
       </c>
@@ -2869,8 +2865,8 @@
       <c r="AA42" s="74"/>
     </row>
     <row r="43" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="90"/>
-      <c r="B43" s="91"/>
+      <c r="A43" s="105"/>
+      <c r="B43" s="106"/>
       <c r="C43" s="17" t="s">
         <v>74</v>
       </c>
@@ -2906,8 +2902,8 @@
       <c r="AA43" s="74"/>
     </row>
     <row r="44" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="90"/>
-      <c r="B44" s="112" t="s">
+      <c r="A44" s="105"/>
+      <c r="B44" s="102" t="s">
         <v>75</v>
       </c>
       <c r="C44" s="17" t="s">
@@ -2945,8 +2941,8 @@
       <c r="AA44" s="74"/>
     </row>
     <row r="45" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="90"/>
-      <c r="B45" s="90"/>
+      <c r="A45" s="105"/>
+      <c r="B45" s="105"/>
       <c r="C45" s="17" t="s">
         <v>77</v>
       </c>
@@ -2982,8 +2978,8 @@
       <c r="AA45" s="74"/>
     </row>
     <row r="46" spans="1:27" s="75" customFormat="1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="91"/>
-      <c r="B46" s="91"/>
+      <c r="A46" s="106"/>
+      <c r="B46" s="106"/>
       <c r="C46" s="17" t="s">
         <v>78</v>
       </c>
@@ -3019,10 +3015,10 @@
       <c r="AA46" s="74"/>
     </row>
     <row r="47" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="107" t="s">
+      <c r="A47" s="97" t="s">
         <v>79</v>
       </c>
-      <c r="B47" s="115" t="s">
+      <c r="B47" s="107" t="s">
         <v>45</v>
       </c>
       <c r="C47" s="17" t="s">
@@ -3060,8 +3056,8 @@
       <c r="AA47" s="1"/>
     </row>
     <row r="48" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="108"/>
-      <c r="B48" s="108"/>
+      <c r="A48" s="98"/>
+      <c r="B48" s="98"/>
       <c r="C48" s="17" t="s">
         <v>81</v>
       </c>
@@ -3097,8 +3093,8 @@
       <c r="AA48" s="1"/>
     </row>
     <row r="49" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="108"/>
-      <c r="B49" s="108"/>
+      <c r="A49" s="98"/>
+      <c r="B49" s="98"/>
       <c r="C49" s="17" t="s">
         <v>82</v>
       </c>
@@ -3134,8 +3130,8 @@
       <c r="AA49" s="1"/>
     </row>
     <row r="50" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="108"/>
-      <c r="B50" s="108"/>
+      <c r="A50" s="98"/>
+      <c r="B50" s="98"/>
       <c r="C50" s="17" t="s">
         <v>83</v>
       </c>
@@ -3171,8 +3167,8 @@
       <c r="AA50" s="1"/>
     </row>
     <row r="51" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="108"/>
-      <c r="B51" s="108"/>
+      <c r="A51" s="98"/>
+      <c r="B51" s="98"/>
       <c r="C51" s="17" t="s">
         <v>84</v>
       </c>
@@ -3208,8 +3204,8 @@
       <c r="AA51" s="1"/>
     </row>
     <row r="52" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="108"/>
-      <c r="B52" s="108"/>
+      <c r="A52" s="98"/>
+      <c r="B52" s="98"/>
       <c r="C52" s="17" t="s">
         <v>85</v>
       </c>
@@ -3245,8 +3241,8 @@
       <c r="AA52" s="1"/>
     </row>
     <row r="53" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="81"/>
-      <c r="B53" s="81"/>
+      <c r="A53" s="83"/>
+      <c r="B53" s="83"/>
       <c r="C53" s="17" t="s">
         <v>86</v>
       </c>
@@ -3282,10 +3278,10 @@
       <c r="AA53" s="1"/>
     </row>
     <row r="54" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="97" t="s">
+      <c r="A54" s="80" t="s">
         <v>87</v>
       </c>
-      <c r="B54" s="95"/>
+      <c r="B54" s="81"/>
       <c r="C54" s="12"/>
       <c r="D54" s="12"/>
       <c r="E54" s="13"/>
@@ -9842,6 +9838,22 @@
     <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="P1:P2"/>
+    <mergeCell ref="Q1:Q2"/>
+    <mergeCell ref="R1:R2"/>
+    <mergeCell ref="S1:S2"/>
+    <mergeCell ref="T1:T2"/>
+    <mergeCell ref="O1:O2"/>
+    <mergeCell ref="A3:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="A20:A23"/>
+    <mergeCell ref="A24:A46"/>
+    <mergeCell ref="D1:D2"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="E1:E2"/>
+    <mergeCell ref="F1:F2"/>
+    <mergeCell ref="G1:N1"/>
     <mergeCell ref="A54:B54"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="B4:B10"/>
@@ -9858,22 +9870,6 @@
     <mergeCell ref="B40:B43"/>
     <mergeCell ref="B44:B46"/>
     <mergeCell ref="B47:B53"/>
-    <mergeCell ref="O1:O2"/>
-    <mergeCell ref="A3:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="A20:A23"/>
-    <mergeCell ref="A24:A46"/>
-    <mergeCell ref="D1:D2"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="E1:E2"/>
-    <mergeCell ref="F1:F2"/>
-    <mergeCell ref="G1:N1"/>
-    <mergeCell ref="P1:P2"/>
-    <mergeCell ref="Q1:Q2"/>
-    <mergeCell ref="R1:R2"/>
-    <mergeCell ref="S1:S2"/>
-    <mergeCell ref="T1:T2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="E3:E53" xr:uid="{00000000-0002-0000-0000-000000000000}">

</xml_diff>